<commit_message>
clear() for arrays added and strings are not 0 terminated anymore
</commit_message>
<xml_diff>
--- a/peddle_tasks.xlsx
+++ b/peddle_tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huebi/workspaces/c64/peddle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE95F7BC-C490-A542-93EB-79C90D0378B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C790E061-B649-1149-A366-C230A32B71F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19280" yWindow="620" windowWidth="47780" windowHeight="22540" xr2:uid="{4C3981A2-71A4-EC48-BDAA-6622CD2AA254}"/>
+    <workbookView xWindow="24420" yWindow="680" windowWidth="47780" windowHeight="22540" activeTab="2" xr2:uid="{4C3981A2-71A4-EC48-BDAA-6622CD2AA254}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,12 @@
   </sheets>
   <definedNames>
     <definedName name="_1.1">Settings!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tasks!$D$1:$D$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tasks!$D$1:$D$52</definedName>
     <definedName name="STATUS">Settings!$A$2:$A$5</definedName>
     <definedName name="tbl_priority">Settings!$D$2:$D$4</definedName>
     <definedName name="tbl_statistics">Statistics!$D$9:$E$9</definedName>
     <definedName name="tbl_type">Settings!$C$2:$C$8</definedName>
-    <definedName name="tbl_version">Settings!$B$2:$B$3</definedName>
+    <definedName name="tbl_version">Settings!$B$2:$B$5</definedName>
     <definedName name="VERSION">Settings!$B$16:$B$1000011</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
   <si>
     <t>Issue No.</t>
   </si>
@@ -129,9 +129,6 @@
     <t>Feature</t>
   </si>
   <si>
-    <t>1.0 (MS1)</t>
-  </si>
-  <si>
     <t>Feedback</t>
   </si>
   <si>
@@ -223,6 +220,54 @@
   </si>
   <si>
     <t>20260505-2</t>
+  </si>
+  <si>
+    <t>struct pointers in function param</t>
+  </si>
+  <si>
+    <t>multiple definitions</t>
+  </si>
+  <si>
+    <t>var x,y,z: int</t>
+  </si>
+  <si>
+    <t>clear() to clear an array</t>
+  </si>
+  <si>
+    <t>play a sound file</t>
+  </si>
+  <si>
+    <t>read from a file on disk</t>
+  </si>
+  <si>
+    <t>communication to internet</t>
+  </si>
+  <si>
+    <t>connect, send, recv, disconnect, available</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>function we don’t need are not in PRG</t>
+  </si>
+  <si>
+    <t>Screen funcs</t>
+  </si>
+  <si>
+    <t>cls(), put(), puts().</t>
+  </si>
+  <si>
+    <t>Dynamic Arrays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">make() creates a dynamic sized array. </t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>1.0</t>
   </si>
 </sst>
 </file>
@@ -447,7 +492,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -593,6 +638,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2278,8 +2324,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}" name="tbl_tasks" displayName="tbl_tasks" ref="A10:N12" totalsRowShown="0" headerRowDxfId="29" headerRowCellStyle="Normal">
-  <autoFilter ref="A10:N12" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}" name="tbl_tasks" displayName="tbl_tasks" ref="A10:N19" totalsRowShown="0" headerRowDxfId="29" headerRowCellStyle="Normal">
+  <autoFilter ref="A10:N19" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{3A74B975-3B34-0646-901A-2D5E3C37739A}" name="Issue No." dataDxfId="28"/>
     <tableColumn id="2" xr3:uid="{B3DF4189-9BAB-D44B-88D8-5094D007655F}" name="Domain" dataDxfId="27"/>
@@ -2327,8 +2373,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}" name="Table1" displayName="Table1" ref="B1:B3" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="B1:B3" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}" name="Table1" displayName="Table1" ref="B1:B5" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="B1:B5" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{BEF8388A-5A10-054C-8B70-FB7ED36EF5DA}" name="Version" dataDxfId="13" dataCellStyle="Normal"/>
   </tableColumns>
@@ -2664,7 +2710,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{232762C2-46AD-F44D-8F38-8855EC80B504}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19" style="24" customWidth="1"/>
@@ -2683,7 +2729,7 @@
   <sheetData>
     <row r="1" spans="1:14" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H1" s="11"/>
       <c r="I1" s="11"/>
@@ -2698,34 +2744,34 @@
     </row>
     <row r="3" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F3" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="H3" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="I3" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="K3" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>50</v>
-      </c>
       <c r="L3" s="17">
-        <f>G13+G15+G17+G18+G20+G19+G21+G22+G24+G35+G36+G42+G46</f>
+        <f>G20+G22+G24+G25+G27+G26+G28+G29+G31+G42+G43+G49+G53</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="C4" s="47" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E4" s="32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F4" s="51">
         <f>SUMIFS(tbl_tasks[Estimation], tbl_tasks[Version], C4)</f>
@@ -2769,12 +2815,12 @@
         <f>COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A2)
  +COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A4)
  +COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A5)</f>
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="E5" s="32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F5" s="51">
         <f>SUMIFS(tbl_tasks[Effort], tbl_tasks[Version], C4)</f>
@@ -2799,16 +2845,16 @@
     </row>
     <row r="6" spans="1:14" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C6" s="46" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="32"/>
       <c r="G6" s="31"/>
       <c r="J6" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K6" s="33">
         <f>K4+K5</f>
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="23" thickBot="1" x14ac:dyDescent="0.25">
@@ -2817,7 +2863,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="58" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F7" s="59">
         <f>1-H4/F4</f>
@@ -2833,16 +2879,16 @@
     </row>
     <row r="9" spans="1:14" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="43" t="s">
-        <v>44</v>
-      </c>
       <c r="G9" s="43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H9" s="43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:14" s="30" customFormat="1" ht="21" x14ac:dyDescent="0.25">
@@ -2859,16 +2905,16 @@
         <v>10</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F10" s="30" t="s">
         <v>2</v>
       </c>
       <c r="G10" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" s="30" t="s">
         <v>32</v>
-      </c>
-      <c r="H10" s="30" t="s">
-        <v>33</v>
       </c>
       <c r="I10" s="30" t="s">
         <v>14</v>
@@ -2891,11 +2937,11 @@
     </row>
     <row r="11" spans="1:14" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E11" s="26"/>
       <c r="F11" s="5" t="s">
@@ -2916,14 +2962,19 @@
       <c r="K11" s="10" t="s">
         <v>4</v>
       </c>
+      <c r="L11" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="M11" s="6"/>
     </row>
-    <row r="12" spans="1:14" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" s="5" customFormat="1" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C12" s="8"/>
-      <c r="D12" s="26"/>
+      <c r="D12" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E12" s="26"/>
       <c r="F12" s="5" t="s">
         <v>12</v>
@@ -2939,116 +2990,186 @@
       <c r="K12" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-    </row>
-    <row r="13" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="L12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="8"/>
-      <c r="D13" s="26"/>
+      <c r="D13" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E13" s="26"/>
       <c r="F13" s="5"/>
       <c r="G13" s="49"/>
       <c r="H13" s="49"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="6"/>
+      <c r="K13" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>61</v>
+      </c>
       <c r="M13" s="6"/>
       <c r="N13" s="5"/>
     </row>
-    <row r="14" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="8"/>
-      <c r="D14" s="26"/>
+      <c r="D14" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E14" s="26"/>
       <c r="F14" s="5"/>
       <c r="G14" s="49"/>
       <c r="H14" s="49"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="6"/>
+      <c r="K14" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="M14" s="6"/>
-    </row>
-    <row r="15" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="N14" s="5"/>
+    </row>
+    <row r="15" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
       <c r="B15" s="5"/>
       <c r="C15" s="8"/>
-      <c r="D15" s="26"/>
+      <c r="D15" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E15" s="26"/>
       <c r="F15" s="5"/>
       <c r="G15" s="49"/>
       <c r="H15" s="49"/>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="6"/>
+      <c r="K15" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="M15" s="6"/>
-    </row>
-    <row r="16" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="N15" s="5"/>
+    </row>
+    <row r="16" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A16" s="4"/>
       <c r="B16" s="5"/>
       <c r="C16" s="8"/>
-      <c r="D16" s="26"/>
+      <c r="D16" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E16" s="26"/>
       <c r="F16" s="5"/>
       <c r="G16" s="49"/>
       <c r="H16" s="49"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
-    </row>
-    <row r="17" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="K16" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="N16" s="5"/>
+    </row>
+    <row r="17" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A17" s="4"/>
       <c r="B17" s="5"/>
       <c r="C17" s="8"/>
-      <c r="D17" s="26"/>
+      <c r="D17" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E17" s="26"/>
       <c r="F17" s="5"/>
       <c r="G17" s="49"/>
       <c r="H17" s="49"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="6"/>
+      <c r="I17" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="M17" s="6"/>
-    </row>
-    <row r="18" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="N17" s="5"/>
+    </row>
+    <row r="18" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A18" s="4"/>
       <c r="B18" s="5"/>
       <c r="C18" s="8"/>
-      <c r="D18" s="26"/>
+      <c r="D18" s="26" t="s">
+        <v>56</v>
+      </c>
       <c r="E18" s="26"/>
       <c r="F18" s="5"/>
       <c r="G18" s="49"/>
       <c r="H18" s="49"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-    </row>
-    <row r="19" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I18" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="N18" s="5"/>
+    </row>
+    <row r="19" spans="1:14" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
       <c r="B19" s="5"/>
       <c r="C19" s="8"/>
-      <c r="D19" s="26"/>
+      <c r="D19" s="26" t="s">
+        <v>66</v>
+      </c>
       <c r="E19" s="26"/>
       <c r="F19" s="5"/>
       <c r="G19" s="49"/>
       <c r="H19" s="49"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
-    </row>
-    <row r="20" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="I19" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="N19" s="5"/>
+    </row>
+    <row r="20" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A20" s="4"/>
       <c r="B20" s="5"/>
       <c r="C20" s="8"/>
@@ -3062,8 +3183,9 @@
       <c r="K20" s="10"/>
       <c r="L20" s="6"/>
       <c r="M20" s="6"/>
-    </row>
-    <row r="21" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="N20" s="5"/>
+    </row>
+    <row r="21" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A21" s="4"/>
       <c r="B21" s="5"/>
       <c r="C21" s="8"/>
@@ -3078,7 +3200,7 @@
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
     </row>
-    <row r="22" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
       <c r="B22" s="5"/>
       <c r="C22" s="8"/>
@@ -3093,7 +3215,7 @@
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>
     </row>
-    <row r="23" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A23" s="4"/>
       <c r="B23" s="5"/>
       <c r="C23" s="8"/>
@@ -3108,7 +3230,7 @@
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
     </row>
-    <row r="24" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
       <c r="B24" s="5"/>
       <c r="C24" s="8"/>
@@ -3123,7 +3245,7 @@
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
     </row>
-    <row r="25" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
       <c r="B25" s="5"/>
       <c r="C25" s="8"/>
@@ -3138,7 +3260,7 @@
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
     </row>
-    <row r="26" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="5"/>
       <c r="C26" s="8"/>
@@ -3153,7 +3275,7 @@
       <c r="L26" s="6"/>
       <c r="M26" s="6"/>
     </row>
-    <row r="27" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="8"/>
@@ -3168,52 +3290,52 @@
       <c r="L27" s="6"/>
       <c r="M27" s="6"/>
     </row>
-    <row r="28" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="5"/>
       <c r="C28" s="8"/>
       <c r="D28" s="26"/>
       <c r="E28" s="26"/>
       <c r="F28" s="5"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
       <c r="I28" s="13"/>
       <c r="J28" s="13"/>
       <c r="K28" s="10"/>
       <c r="L28" s="6"/>
       <c r="M28" s="6"/>
     </row>
-    <row r="29" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="5"/>
       <c r="C29" s="8"/>
       <c r="D29" s="26"/>
       <c r="E29" s="26"/>
       <c r="F29" s="5"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="49"/>
       <c r="I29" s="13"/>
       <c r="J29" s="13"/>
       <c r="K29" s="10"/>
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
     </row>
-    <row r="30" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A30" s="4"/>
       <c r="B30" s="5"/>
       <c r="C30" s="8"/>
       <c r="D30" s="26"/>
       <c r="E30" s="26"/>
       <c r="F30" s="5"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
+      <c r="G30" s="49"/>
+      <c r="H30" s="49"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="10"/>
       <c r="L30" s="6"/>
       <c r="M30" s="6"/>
     </row>
-    <row r="31" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A31" s="4"/>
       <c r="B31" s="5"/>
       <c r="C31" s="8"/>
@@ -3228,7 +3350,7 @@
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
     </row>
-    <row r="32" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A32" s="4"/>
       <c r="B32" s="5"/>
       <c r="C32" s="8"/>
@@ -3265,8 +3387,8 @@
       <c r="D34" s="26"/>
       <c r="E34" s="26"/>
       <c r="F34" s="5"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
+      <c r="G34" s="49"/>
+      <c r="H34" s="49"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
       <c r="K34" s="10"/>
@@ -3280,8 +3402,8 @@
       <c r="D35" s="26"/>
       <c r="E35" s="26"/>
       <c r="F35" s="5"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
       <c r="I35" s="13"/>
       <c r="J35" s="13"/>
       <c r="K35" s="10"/>
@@ -3295,8 +3417,8 @@
       <c r="D36" s="26"/>
       <c r="E36" s="26"/>
       <c r="F36" s="5"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
       <c r="I36" s="13"/>
       <c r="J36" s="13"/>
       <c r="K36" s="10"/>
@@ -3310,8 +3432,8 @@
       <c r="D37" s="26"/>
       <c r="E37" s="26"/>
       <c r="F37" s="5"/>
-      <c r="G37" s="49"/>
-      <c r="H37" s="49"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
       <c r="I37" s="13"/>
       <c r="J37" s="13"/>
       <c r="K37" s="10"/>
@@ -3370,8 +3492,8 @@
       <c r="D41" s="26"/>
       <c r="E41" s="26"/>
       <c r="F41" s="5"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
       <c r="I41" s="13"/>
       <c r="J41" s="13"/>
       <c r="K41" s="10"/>
@@ -3400,8 +3522,8 @@
       <c r="D43" s="26"/>
       <c r="E43" s="26"/>
       <c r="F43" s="5"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
+      <c r="G43" s="49"/>
+      <c r="H43" s="49"/>
       <c r="I43" s="13"/>
       <c r="J43" s="13"/>
       <c r="K43" s="10"/>
@@ -3415,8 +3537,8 @@
       <c r="D44" s="26"/>
       <c r="E44" s="26"/>
       <c r="F44" s="5"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13"/>
+      <c r="G44" s="49"/>
+      <c r="H44" s="49"/>
       <c r="I44" s="13"/>
       <c r="J44" s="13"/>
       <c r="K44" s="10"/>
@@ -3490,8 +3612,8 @@
       <c r="D49" s="26"/>
       <c r="E49" s="26"/>
       <c r="F49" s="5"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
+      <c r="G49" s="49"/>
+      <c r="H49" s="49"/>
       <c r="I49" s="13"/>
       <c r="J49" s="13"/>
       <c r="K49" s="10"/>
@@ -3535,8 +3657,8 @@
       <c r="D52" s="26"/>
       <c r="E52" s="26"/>
       <c r="F52" s="5"/>
-      <c r="G52" s="13"/>
-      <c r="H52" s="13"/>
+      <c r="G52" s="49"/>
+      <c r="H52" s="49"/>
       <c r="I52" s="13"/>
       <c r="J52" s="13"/>
       <c r="K52" s="10"/>
@@ -3550,8 +3672,8 @@
       <c r="D53" s="26"/>
       <c r="E53" s="26"/>
       <c r="F53" s="5"/>
-      <c r="G53" s="13"/>
-      <c r="H53" s="13"/>
+      <c r="G53" s="49"/>
+      <c r="H53" s="49"/>
       <c r="I53" s="13"/>
       <c r="J53" s="13"/>
       <c r="K53" s="10"/>
@@ -3565,8 +3687,8 @@
       <c r="D54" s="26"/>
       <c r="E54" s="26"/>
       <c r="F54" s="5"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
+      <c r="G54" s="49"/>
+      <c r="H54" s="49"/>
       <c r="I54" s="13"/>
       <c r="J54" s="13"/>
       <c r="K54" s="10"/>
@@ -3580,8 +3702,8 @@
       <c r="D55" s="26"/>
       <c r="E55" s="26"/>
       <c r="F55" s="5"/>
-      <c r="G55" s="13"/>
-      <c r="H55" s="13"/>
+      <c r="G55" s="49"/>
+      <c r="H55" s="49"/>
       <c r="I55" s="13"/>
       <c r="J55" s="13"/>
       <c r="K55" s="10"/>
@@ -3617,7 +3739,6 @@
       <c r="K57" s="10"/>
       <c r="L57" s="6"/>
       <c r="M57" s="6"/>
-      <c r="N57" s="60"/>
     </row>
     <row r="58" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A58" s="4"/>
@@ -3723,6 +3844,7 @@
       <c r="K64" s="10"/>
       <c r="L64" s="6"/>
       <c r="M64" s="6"/>
+      <c r="N64" s="60"/>
     </row>
     <row r="65" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A65" s="4"/>
@@ -3904,14 +4026,119 @@
       <c r="L76" s="6"/>
       <c r="M76" s="6"/>
     </row>
+    <row r="77" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A77" s="4"/>
+      <c r="B77" s="5"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="26"/>
+      <c r="E77" s="26"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="13"/>
+      <c r="H77" s="13"/>
+      <c r="I77" s="13"/>
+      <c r="J77" s="13"/>
+      <c r="K77" s="10"/>
+      <c r="L77" s="6"/>
+      <c r="M77" s="6"/>
+    </row>
+    <row r="78" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A78" s="4"/>
+      <c r="B78" s="5"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="26"/>
+      <c r="E78" s="26"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="13"/>
+      <c r="H78" s="13"/>
+      <c r="I78" s="13"/>
+      <c r="J78" s="13"/>
+      <c r="K78" s="10"/>
+      <c r="L78" s="6"/>
+      <c r="M78" s="6"/>
+    </row>
+    <row r="79" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A79" s="4"/>
+      <c r="B79" s="5"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="13"/>
+      <c r="H79" s="13"/>
+      <c r="I79" s="13"/>
+      <c r="J79" s="13"/>
+      <c r="K79" s="10"/>
+      <c r="L79" s="6"/>
+      <c r="M79" s="6"/>
+    </row>
+    <row r="80" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A80" s="4"/>
+      <c r="B80" s="5"/>
+      <c r="C80" s="8"/>
+      <c r="D80" s="26"/>
+      <c r="E80" s="26"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="13"/>
+      <c r="H80" s="13"/>
+      <c r="I80" s="13"/>
+      <c r="J80" s="13"/>
+      <c r="K80" s="10"/>
+      <c r="L80" s="6"/>
+      <c r="M80" s="6"/>
+    </row>
+    <row r="81" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A81" s="4"/>
+      <c r="B81" s="5"/>
+      <c r="C81" s="8"/>
+      <c r="D81" s="26"/>
+      <c r="E81" s="26"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="13"/>
+      <c r="H81" s="13"/>
+      <c r="I81" s="13"/>
+      <c r="J81" s="13"/>
+      <c r="K81" s="10"/>
+      <c r="L81" s="6"/>
+      <c r="M81" s="6"/>
+    </row>
+    <row r="82" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A82" s="4"/>
+      <c r="B82" s="5"/>
+      <c r="C82" s="8"/>
+      <c r="D82" s="26"/>
+      <c r="E82" s="26"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="13"/>
+      <c r="H82" s="13"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="13"/>
+      <c r="K82" s="10"/>
+      <c r="L82" s="6"/>
+      <c r="M82" s="6"/>
+    </row>
+    <row r="83" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A83" s="4"/>
+      <c r="B83" s="5"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="26"/>
+      <c r="E83" s="26"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="13"/>
+      <c r="H83" s="13"/>
+      <c r="I83" s="13"/>
+      <c r="J83" s="13"/>
+      <c r="K83" s="10"/>
+      <c r="L83" s="6"/>
+      <c r="M83" s="6"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="I11:I12">
+  <conditionalFormatting sqref="I11:I19">
     <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"Investigation"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:J2 J77:J1048576 K10:K12">
+  <conditionalFormatting sqref="J1:J2 J84:J1048576 K10:K19">
     <cfRule type="containsText" dxfId="3" priority="1" stopIfTrue="1" operator="containsText" text="CRITICAL">
       <formula>NOT(ISERROR(SEARCH("CRITICAL",J1)))</formula>
     </cfRule>
@@ -3926,16 +4153,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F77:G1048576 J77:J1048576 C4 D11:D1048576 E11:E76" xr:uid="{A96B27E9-62CD-6847-959C-A801683B206F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F84:G1048576 J84:J1048576 C4 E11:E83 D11:D1048576" xr:uid="{A96B27E9-62CD-6847-959C-A801683B206F}">
       <formula1>tbl_version</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J77:J1048576 K11:K76" xr:uid="{E9C1BB5C-3BBC-2D45-ABAA-9307D27F88B9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J84:J1048576 K11:K83" xr:uid="{E9C1BB5C-3BBC-2D45-ABAA-9307D27F88B9}">
       <formula1>STATUS</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H77:H1048576 I11:I12" xr:uid="{647DF7B9-149A-044D-BE08-FED4FA7A1001}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H84:H1048576 I11:I19" xr:uid="{647DF7B9-149A-044D-BE08-FED4FA7A1001}">
       <formula1>tbl_type</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I77:I1048576 J11:J12" xr:uid="{C452C5EF-EF77-304A-B117-32B247EEAD4B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I84:I1048576 J11:J19" xr:uid="{C452C5EF-EF77-304A-B117-32B247EEAD4B}">
       <formula1>tbl_priority</formula1>
     </dataValidation>
   </dataValidations>
@@ -3970,12 +4197,12 @@
         <v>24</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C3" s="48" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" s="18">
         <v>46147</v>
@@ -3985,7 +4212,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J3" s="35"/>
       <c r="K3" s="35"/>
@@ -4000,7 +4227,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C4" s="29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="18" t="e">
         <f>-INTERCEPT(E9:E9,D9:D9)/SLOPE(E9:E9,D9:D9)</f>
@@ -4010,7 +4237,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J4" s="38"/>
       <c r="K4" s="38"/>
@@ -4025,7 +4252,7 @@
     </row>
     <row r="5" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="I5" s="40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J5" s="41"/>
       <c r="K5" s="41"/>
@@ -4046,17 +4273,17 @@
         <v>23</v>
       </c>
       <c r="F6" s="54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G6" s="54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C7"/>
       <c r="D7" s="55">
         <f ca="1">TODAY()</f>
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="E7" s="56">
         <f>Tasks!H4</f>
@@ -4064,11 +4291,11 @@
       </c>
       <c r="F7" s="57">
         <f>Tasks!K6</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G7" s="57">
         <f>Tasks!K4</f>
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
@@ -4077,13 +4304,13 @@
         <v>24</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
@@ -4235,7 +4462,7 @@
         <v>18</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G1" s="53">
         <v>8</v>
@@ -4246,7 +4473,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -4259,8 +4486,8 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>27</v>
+      <c r="B3" s="61" t="s">
+        <v>66</v>
       </c>
       <c r="C3" t="s">
         <v>16</v>
@@ -4273,6 +4500,9 @@
       <c r="A4" t="s">
         <v>9</v>
       </c>
+      <c r="B4" s="61" t="s">
+        <v>73</v>
+      </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
@@ -4282,7 +4512,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
@@ -4295,12 +4528,12 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
timers added, joystick example added
</commit_message>
<xml_diff>
--- a/peddle_tasks.xlsx
+++ b/peddle_tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huebi/workspaces/c64/peddle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78369921-1C54-1E44-9B6B-827BD756B3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BA4EB1-E6CE-1243-9FD9-009198687672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24420" yWindow="680" windowWidth="47780" windowHeight="22540" xr2:uid="{4C3981A2-71A4-EC48-BDAA-6622CD2AA254}"/>
+    <workbookView xWindow="21020" yWindow="680" windowWidth="47780" windowHeight="22540" xr2:uid="{4C3981A2-71A4-EC48-BDAA-6622CD2AA254}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_1.1">Settings!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tasks!$D$1:$D$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tasks!$D$1:$D$57</definedName>
     <definedName name="STATUS">Settings!$A$2:$A$5</definedName>
     <definedName name="tbl_priority">Settings!$D$2:$D$4</definedName>
     <definedName name="tbl_statistics">Statistics!$D$9:$E$9</definedName>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="82">
   <si>
     <t>Issue No.</t>
   </si>
@@ -222,9 +222,6 @@
     <t>20260505-2</t>
   </si>
   <si>
-    <t>struct pointers in function param</t>
-  </si>
-  <si>
     <t>multiple definitions</t>
   </si>
   <si>
@@ -286,6 +283,15 @@
   </si>
   <si>
     <t>add Hexnumber prefix 0x</t>
+  </si>
+  <si>
+    <t>pointer params</t>
+  </si>
+  <si>
+    <t>20260524-1</t>
+  </si>
+  <si>
+    <t>for loop</t>
   </si>
 </sst>
 </file>
@@ -510,7 +516,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -655,120 +661,12 @@
     <xf numFmtId="9" fontId="9" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="34">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00FA00"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF2600"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="29">
     <dxf>
       <font>
         <color theme="0"/>
@@ -937,6 +835,18 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
     </dxf>
     <dxf>
       <font>
@@ -1201,18 +1111,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2342,8 +2240,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}" name="tbl_tasks" displayName="tbl_tasks" ref="A10:N22" totalsRowShown="0" headerRowDxfId="29" headerRowCellStyle="Normal">
-  <autoFilter ref="A10:N22" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}" name="tbl_tasks" displayName="tbl_tasks" ref="A10:N24" totalsRowShown="0" headerRowDxfId="28" headerRowCellStyle="Normal">
+  <autoFilter ref="A10:N24" xr:uid="{0C49DA46-06FF-584F-9195-6A87344D314F}">
     <filterColumn colId="10">
       <filters>
         <filter val="OPEN"/>
@@ -2351,19 +2249,19 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{3A74B975-3B34-0646-901A-2D5E3C37739A}" name="Issue No." dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{B3DF4189-9BAB-D44B-88D8-5094D007655F}" name="Domain" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{17A7DA6B-442B-C244-8FAE-6256230CA506}" name="Due Date" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{1F8EA6E5-C966-6941-BB9C-8BC47017CBC2}" name="Version" dataDxfId="25"/>
-    <tableColumn id="14" xr3:uid="{0EBAADC4-5639-434C-90BA-03CDB29B20BB}" name="Implemented" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{CF3F8B3C-43C7-0B4F-80D2-28EE285FF6C0}" name="Responsible" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{CCF59F26-1875-6148-8023-44891473DDA4}" name="Estimation" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{FDCB0EA8-E1F8-6442-8410-58449391FECC}" name="Effort" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{C67CF053-5D1A-3E40-B474-3B6C57565CF1}" name="Type" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{42C03962-A72B-ED4E-8A41-477E05EB937A}" name="Priority" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{5A9CF61C-B8F5-D244-BED8-93D82BB47F76}" name="Status" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{3AAE5B09-F591-D645-9E17-09E63C663002}" name="Issue" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{E117AD2F-3CDB-A946-A5DB-FCE15FAD0D2F}" name="Description" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{3A74B975-3B34-0646-901A-2D5E3C37739A}" name="Issue No." dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{B3DF4189-9BAB-D44B-88D8-5094D007655F}" name="Domain" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{17A7DA6B-442B-C244-8FAE-6256230CA506}" name="Due Date" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{1F8EA6E5-C966-6941-BB9C-8BC47017CBC2}" name="Version" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{0EBAADC4-5639-434C-90BA-03CDB29B20BB}" name="Implemented" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{CF3F8B3C-43C7-0B4F-80D2-28EE285FF6C0}" name="Responsible" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{CCF59F26-1875-6148-8023-44891473DDA4}" name="Estimation" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{FDCB0EA8-E1F8-6442-8410-58449391FECC}" name="Effort" dataDxfId="20"/>
+    <tableColumn id="8" xr3:uid="{C67CF053-5D1A-3E40-B474-3B6C57565CF1}" name="Type" dataDxfId="19"/>
+    <tableColumn id="9" xr3:uid="{42C03962-A72B-ED4E-8A41-477E05EB937A}" name="Priority" dataDxfId="18"/>
+    <tableColumn id="10" xr3:uid="{5A9CF61C-B8F5-D244-BED8-93D82BB47F76}" name="Status" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{3AAE5B09-F591-D645-9E17-09E63C663002}" name="Issue" dataDxfId="16"/>
+    <tableColumn id="12" xr3:uid="{E117AD2F-3CDB-A946-A5DB-FCE15FAD0D2F}" name="Description" dataDxfId="15"/>
     <tableColumn id="13" xr3:uid="{415555C1-82CD-2B43-B211-238CF178048D}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2374,10 +2272,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3D0ACB0F-D554-B542-8779-C2951F9CB2E3}" name="tbl_stats" displayName="tbl_stats" ref="D8:G9" totalsRowShown="0">
   <autoFilter ref="D8:G9" xr:uid="{3D0ACB0F-D554-B542-8779-C2951F9CB2E3}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{32BE3B30-9560-D44E-9507-53A1DF9C7BFA}" name="Date" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{8EB8D535-33FB-9840-9ABA-39B2CA617B39}" name="Estimation" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{379141BC-2C5D-5644-A94D-E20C699E4B47}" name="Tasks" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{4690FA52-52AA-B04B-B16D-7AFE9079CD30}" name="OpenTasks" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{32BE3B30-9560-D44E-9507-53A1DF9C7BFA}" name="Date" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{8EB8D535-33FB-9840-9ABA-39B2CA617B39}" name="Estimation" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{379141BC-2C5D-5644-A94D-E20C699E4B47}" name="Tasks" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{4690FA52-52AA-B04B-B16D-7AFE9079CD30}" name="OpenTasks" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2397,17 +2295,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}" name="Table1" displayName="Table1" ref="B1:B5" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}" name="Table1" displayName="Table1" ref="B1:B5" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="B1:B5" xr:uid="{93345991-FEF1-9246-AEF9-D40B5350E6C7}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{BEF8388A-5A10-054C-8B70-FB7ED36EF5DA}" name="Version" dataDxfId="13" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{BEF8388A-5A10-054C-8B70-FB7ED36EF5DA}" name="Version" dataDxfId="8" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8E52021A-A2D1-654C-A028-4B6E5BD9B9C8}" name="Table2" displayName="Table2" ref="C1:C8" totalsRowShown="0" headerRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8E52021A-A2D1-654C-A028-4B6E5BD9B9C8}" name="Table2" displayName="Table2" ref="C1:C8" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="C1:C8" xr:uid="{8E52021A-A2D1-654C-A028-4B6E5BD9B9C8}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{8B2A05F6-B05E-304D-B64A-3E7ACDFD1BF6}" name="Type"/>
@@ -2417,7 +2315,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2446FBF7-B40E-294F-BD51-C6A3ABB9CD6F}" name="Table3" displayName="Table3" ref="D1:D4" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2446FBF7-B40E-294F-BD51-C6A3ABB9CD6F}" name="Table3" displayName="Table3" ref="D1:D4" totalsRowShown="0" headerRowDxfId="6">
   <autoFilter ref="D1:D4" xr:uid="{2446FBF7-B40E-294F-BD51-C6A3ABB9CD6F}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{62C2997E-BA07-7A4F-8344-735015F39C17}" name="Priority"/>
@@ -2427,7 +2325,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{518AFD7F-84E2-C945-86A4-ABC13F78B0EF}" name="Table6" displayName="Table6" ref="A1:A5" totalsRowShown="0" headerRowDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{518AFD7F-84E2-C945-86A4-ABC13F78B0EF}" name="Table6" displayName="Table6" ref="A1:A5" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:A5" xr:uid="{518AFD7F-84E2-C945-86A4-ABC13F78B0EF}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{7F0FB6F0-A736-454A-BEEF-7787535BD26D}" name="Status"/>
@@ -2734,7 +2632,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{232762C2-46AD-F44D-8F38-8855EC80B504}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19" style="24" customWidth="1"/>
@@ -2786,7 +2684,7 @@
         <v>49</v>
       </c>
       <c r="L3" s="17">
-        <f>G23+G25+G27+G28+G30+G29+G31+G32+G34+G45+G46+G52+G56</f>
+        <f>G25+G27+G29+G30+G32+G31+G33+G34+G36+G47+G48+G54+G58</f>
         <v>0</v>
       </c>
     </row>
@@ -2839,7 +2737,7 @@
         <f>COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A2)
  +COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A4)
  +COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A5)</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="20" x14ac:dyDescent="0.2">
@@ -2864,7 +2762,7 @@
       </c>
       <c r="K5" s="20">
         <f>COUNTIFS(tbl_tasks[Version],C4,tbl_tasks[Status],Settings!A3)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="20" thickBot="1" x14ac:dyDescent="0.25">
@@ -2987,7 +2885,7 @@
         <v>4</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="M11" s="6"/>
     </row>
@@ -3015,10 +2913,10 @@
         <v>8</v>
       </c>
       <c r="L12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M12" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="20" hidden="1" x14ac:dyDescent="0.2">
@@ -3038,7 +2936,7 @@
         <v>8</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M13" s="6"/>
       <c r="N13" s="5"/>
@@ -3060,7 +2958,7 @@
         <v>4</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M14" s="6"/>
       <c r="N14" s="5"/>
@@ -3082,7 +2980,7 @@
         <v>4</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M15" s="6"/>
       <c r="N15" s="5"/>
@@ -3104,10 +3002,10 @@
         <v>4</v>
       </c>
       <c r="L16" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M16" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="N16" s="5"/>
     </row>
@@ -3132,7 +3030,7 @@
         <v>8</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M17" s="6"/>
       <c r="N17" s="5"/>
@@ -3155,13 +3053,13 @@
         <v>19</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="M18" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="N18" s="5"/>
     </row>
@@ -3170,7 +3068,7 @@
       <c r="B19" s="5"/>
       <c r="C19" s="8"/>
       <c r="D19" s="26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E19" s="26"/>
       <c r="F19" s="5"/>
@@ -3186,10 +3084,10 @@
         <v>4</v>
       </c>
       <c r="L19" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="M19" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>71</v>
       </c>
       <c r="N19" s="5"/>
     </row>
@@ -3214,10 +3112,10 @@
         <v>8</v>
       </c>
       <c r="L20" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M20" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>75</v>
       </c>
       <c r="N20" s="5"/>
     </row>
@@ -3239,13 +3137,13 @@
         <v>19</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L21" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="M21" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="N21" s="5"/>
     </row>
@@ -3267,29 +3165,43 @@
         <v>19</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L22" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="M22" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M22" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="N22" s="5"/>
     </row>
-    <row r="23" spans="1:14" ht="19" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
+    <row r="23" spans="1:14" ht="20" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="B23" s="5"/>
       <c r="C23" s="8"/>
-      <c r="D23" s="26"/>
+      <c r="D23" s="26" t="s">
+        <v>72</v>
+      </c>
       <c r="E23" s="26"/>
-      <c r="F23" s="5"/>
+      <c r="F23" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="G23" s="49"/>
       <c r="H23" s="49"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="6"/>
+      <c r="I23" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K23" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>81</v>
+      </c>
       <c r="M23" s="6"/>
       <c r="N23" s="5"/>
     </row>
@@ -3307,6 +3219,7 @@
       <c r="K24" s="10"/>
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
+      <c r="N24" s="5"/>
     </row>
     <row r="25" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
@@ -3322,6 +3235,7 @@
       <c r="K25" s="10"/>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
+      <c r="N25" s="5"/>
     </row>
     <row r="26" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
@@ -3510,8 +3424,8 @@
       <c r="D38" s="26"/>
       <c r="E38" s="26"/>
       <c r="F38" s="5"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
       <c r="I38" s="13"/>
       <c r="J38" s="13"/>
       <c r="K38" s="10"/>
@@ -3525,8 +3439,8 @@
       <c r="D39" s="26"/>
       <c r="E39" s="26"/>
       <c r="F39" s="5"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="49"/>
       <c r="I39" s="13"/>
       <c r="J39" s="13"/>
       <c r="K39" s="10"/>
@@ -3555,8 +3469,8 @@
       <c r="D41" s="26"/>
       <c r="E41" s="26"/>
       <c r="F41" s="5"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
       <c r="I41" s="13"/>
       <c r="J41" s="13"/>
       <c r="K41" s="10"/>
@@ -3570,8 +3484,8 @@
       <c r="D42" s="26"/>
       <c r="E42" s="26"/>
       <c r="F42" s="5"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
       <c r="I42" s="13"/>
       <c r="J42" s="13"/>
       <c r="K42" s="10"/>
@@ -3600,8 +3514,8 @@
       <c r="D44" s="26"/>
       <c r="E44" s="26"/>
       <c r="F44" s="5"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13"/>
+      <c r="G44" s="49"/>
+      <c r="H44" s="49"/>
       <c r="I44" s="13"/>
       <c r="J44" s="13"/>
       <c r="K44" s="10"/>
@@ -3630,8 +3544,8 @@
       <c r="D46" s="26"/>
       <c r="E46" s="26"/>
       <c r="F46" s="5"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="49"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="13"/>
       <c r="I46" s="13"/>
       <c r="J46" s="13"/>
       <c r="K46" s="10"/>
@@ -3735,8 +3649,8 @@
       <c r="D53" s="26"/>
       <c r="E53" s="26"/>
       <c r="F53" s="5"/>
-      <c r="G53" s="13"/>
-      <c r="H53" s="13"/>
+      <c r="G53" s="49"/>
+      <c r="H53" s="49"/>
       <c r="I53" s="13"/>
       <c r="J53" s="13"/>
       <c r="K53" s="10"/>
@@ -3750,8 +3664,8 @@
       <c r="D54" s="26"/>
       <c r="E54" s="26"/>
       <c r="F54" s="5"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
+      <c r="G54" s="49"/>
+      <c r="H54" s="49"/>
       <c r="I54" s="13"/>
       <c r="J54" s="13"/>
       <c r="K54" s="10"/>
@@ -3765,8 +3679,8 @@
       <c r="D55" s="26"/>
       <c r="E55" s="26"/>
       <c r="F55" s="5"/>
-      <c r="G55" s="49"/>
-      <c r="H55" s="49"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="13"/>
       <c r="I55" s="13"/>
       <c r="J55" s="13"/>
       <c r="K55" s="10"/>
@@ -3780,8 +3694,8 @@
       <c r="D56" s="26"/>
       <c r="E56" s="26"/>
       <c r="F56" s="5"/>
-      <c r="G56" s="49"/>
-      <c r="H56" s="49"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="13"/>
       <c r="I56" s="13"/>
       <c r="J56" s="13"/>
       <c r="K56" s="10"/>
@@ -3825,8 +3739,8 @@
       <c r="D59" s="26"/>
       <c r="E59" s="26"/>
       <c r="F59" s="5"/>
-      <c r="G59" s="13"/>
-      <c r="H59" s="13"/>
+      <c r="G59" s="49"/>
+      <c r="H59" s="49"/>
       <c r="I59" s="13"/>
       <c r="J59" s="13"/>
       <c r="K59" s="10"/>
@@ -3840,8 +3754,8 @@
       <c r="D60" s="26"/>
       <c r="E60" s="26"/>
       <c r="F60" s="5"/>
-      <c r="G60" s="13"/>
-      <c r="H60" s="13"/>
+      <c r="G60" s="49"/>
+      <c r="H60" s="49"/>
       <c r="I60" s="13"/>
       <c r="J60" s="13"/>
       <c r="K60" s="10"/>
@@ -3908,7 +3822,7 @@
       <c r="L64" s="6"/>
       <c r="M64" s="6"/>
     </row>
-    <row r="65" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A65" s="4"/>
       <c r="B65" s="5"/>
       <c r="C65" s="8"/>
@@ -3923,7 +3837,7 @@
       <c r="L65" s="6"/>
       <c r="M65" s="6"/>
     </row>
-    <row r="66" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A66" s="4"/>
       <c r="B66" s="5"/>
       <c r="C66" s="8"/>
@@ -3938,7 +3852,7 @@
       <c r="L66" s="6"/>
       <c r="M66" s="6"/>
     </row>
-    <row r="67" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A67" s="4"/>
       <c r="B67" s="5"/>
       <c r="C67" s="8"/>
@@ -3952,9 +3866,8 @@
       <c r="K67" s="10"/>
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
-      <c r="N67" s="60"/>
-    </row>
-    <row r="68" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="68" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A68" s="4"/>
       <c r="B68" s="5"/>
       <c r="C68" s="8"/>
@@ -3969,7 +3882,7 @@
       <c r="L68" s="6"/>
       <c r="M68" s="6"/>
     </row>
-    <row r="69" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A69" s="4"/>
       <c r="B69" s="5"/>
       <c r="C69" s="8"/>
@@ -3984,7 +3897,7 @@
       <c r="L69" s="6"/>
       <c r="M69" s="6"/>
     </row>
-    <row r="70" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A70" s="4"/>
       <c r="B70" s="5"/>
       <c r="C70" s="8"/>
@@ -3999,7 +3912,7 @@
       <c r="L70" s="6"/>
       <c r="M70" s="6"/>
     </row>
-    <row r="71" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A71" s="4"/>
       <c r="B71" s="5"/>
       <c r="C71" s="8"/>
@@ -4014,7 +3927,7 @@
       <c r="L71" s="6"/>
       <c r="M71" s="6"/>
     </row>
-    <row r="72" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A72" s="4"/>
       <c r="B72" s="5"/>
       <c r="C72" s="8"/>
@@ -4029,7 +3942,7 @@
       <c r="L72" s="6"/>
       <c r="M72" s="6"/>
     </row>
-    <row r="73" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A73" s="4"/>
       <c r="B73" s="5"/>
       <c r="C73" s="8"/>
@@ -4044,7 +3957,7 @@
       <c r="L73" s="6"/>
       <c r="M73" s="6"/>
     </row>
-    <row r="74" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A74" s="4"/>
       <c r="B74" s="5"/>
       <c r="C74" s="8"/>
@@ -4059,7 +3972,7 @@
       <c r="L74" s="6"/>
       <c r="M74" s="6"/>
     </row>
-    <row r="75" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A75" s="4"/>
       <c r="B75" s="5"/>
       <c r="C75" s="8"/>
@@ -4074,7 +3987,7 @@
       <c r="L75" s="6"/>
       <c r="M75" s="6"/>
     </row>
-    <row r="76" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A76" s="4"/>
       <c r="B76" s="5"/>
       <c r="C76" s="8"/>
@@ -4089,7 +4002,7 @@
       <c r="L76" s="6"/>
       <c r="M76" s="6"/>
     </row>
-    <row r="77" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A77" s="4"/>
       <c r="B77" s="5"/>
       <c r="C77" s="8"/>
@@ -4104,7 +4017,7 @@
       <c r="L77" s="6"/>
       <c r="M77" s="6"/>
     </row>
-    <row r="78" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A78" s="4"/>
       <c r="B78" s="5"/>
       <c r="C78" s="8"/>
@@ -4119,7 +4032,7 @@
       <c r="L78" s="6"/>
       <c r="M78" s="6"/>
     </row>
-    <row r="79" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A79" s="4"/>
       <c r="B79" s="5"/>
       <c r="C79" s="8"/>
@@ -4134,7 +4047,7 @@
       <c r="L79" s="6"/>
       <c r="M79" s="6"/>
     </row>
-    <row r="80" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:13" ht="19" x14ac:dyDescent="0.2">
       <c r="A80" s="4"/>
       <c r="B80" s="5"/>
       <c r="C80" s="8"/>
@@ -4239,14 +4152,44 @@
       <c r="L86" s="6"/>
       <c r="M86" s="6"/>
     </row>
+    <row r="87" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A87" s="4"/>
+      <c r="B87" s="5"/>
+      <c r="C87" s="8"/>
+      <c r="D87" s="26"/>
+      <c r="E87" s="26"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="13"/>
+      <c r="H87" s="13"/>
+      <c r="I87" s="13"/>
+      <c r="J87" s="13"/>
+      <c r="K87" s="10"/>
+      <c r="L87" s="6"/>
+      <c r="M87" s="6"/>
+    </row>
+    <row r="88" spans="1:13" ht="19" x14ac:dyDescent="0.2">
+      <c r="A88" s="4"/>
+      <c r="B88" s="5"/>
+      <c r="C88" s="8"/>
+      <c r="D88" s="26"/>
+      <c r="E88" s="26"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="13"/>
+      <c r="H88" s="13"/>
+      <c r="I88" s="13"/>
+      <c r="J88" s="13"/>
+      <c r="K88" s="10"/>
+      <c r="L88" s="6"/>
+      <c r="M88" s="6"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="I11:I22">
+  <conditionalFormatting sqref="I11:I24">
     <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"Investigation"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:J2 J87:J1048576 K10:K22">
+  <conditionalFormatting sqref="J1:J2 J89:J1048576 K10:K24">
     <cfRule type="containsText" dxfId="3" priority="1" stopIfTrue="1" operator="containsText" text="CRITICAL">
       <formula>NOT(ISERROR(SEARCH("CRITICAL",J1)))</formula>
     </cfRule>
@@ -4261,16 +4204,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F87:G1048576 J87:J1048576 C4 D11:D1048576 E11:E86" xr:uid="{A96B27E9-62CD-6847-959C-A801683B206F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F89:G1048576 J89:J1048576 C4 D11:D1048576 E11:E88" xr:uid="{A96B27E9-62CD-6847-959C-A801683B206F}">
       <formula1>tbl_version</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J87:J1048576 K11:K86" xr:uid="{E9C1BB5C-3BBC-2D45-ABAA-9307D27F88B9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J89:J1048576 K11:K88" xr:uid="{E9C1BB5C-3BBC-2D45-ABAA-9307D27F88B9}">
       <formula1>STATUS</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H87:H1048576 I11:I22" xr:uid="{647DF7B9-149A-044D-BE08-FED4FA7A1001}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H89:H1048576 I11:I24" xr:uid="{647DF7B9-149A-044D-BE08-FED4FA7A1001}">
       <formula1>tbl_type</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I87:I1048576 J11:J22" xr:uid="{C452C5EF-EF77-304A-B117-32B247EEAD4B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I89:I1048576 J11:J24" xr:uid="{C452C5EF-EF77-304A-B117-32B247EEAD4B}">
       <formula1>tbl_priority</formula1>
     </dataValidation>
   </dataValidations>
@@ -4391,7 +4334,7 @@
       <c r="C7"/>
       <c r="D7" s="55">
         <f ca="1">TODAY()</f>
-        <v>46149</v>
+        <v>46166</v>
       </c>
       <c r="E7" s="56">
         <f>Tasks!H4</f>
@@ -4403,7 +4346,7 @@
       </c>
       <c r="G7" s="57">
         <f>Tasks!K4</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
@@ -4594,8 +4537,8 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="61" t="s">
-        <v>66</v>
+      <c r="B3" s="15" t="s">
+        <v>65</v>
       </c>
       <c r="C3" t="s">
         <v>16</v>
@@ -4608,8 +4551,8 @@
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="61" t="s">
-        <v>73</v>
+      <c r="B4" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -4623,7 +4566,7 @@
         <v>30</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>

</xml_diff>